<commit_message>
feat: implement core application architecture with UI widgets, serial communication, and decoder modules
</commit_message>
<xml_diff>
--- a/single cell configuration.xlsx
+++ b/single cell configuration.xlsx
@@ -474,97 +474,97 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>profile_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>parser_type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>header_hex</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>frame_id_size</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>frame_id_byte_order</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>length_size</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>length_meaning</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>length_byte_order</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>crc_type</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>crc_size</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>crc_byte_order</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>crc_coverage</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>footer_hex</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>escape_mode</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>raw_log_format</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>inter_frame_delay_ms</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>tx_pad_length</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>modbus_node_address</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>single cell configuration</t>
+          <t>Experiment 1 Single Cell BMS</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -623,14 +623,13 @@
       <c r="P2" t="n">
         <v>10</v>
       </c>
-      <c r="Q2" t="n">
-        <v>12</v>
-      </c>
       <c r="R2" t="n">
         <v>1</v>
       </c>
-      <c r="S2" t="b">
-        <v>1</v>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -704,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8.36328125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -716,32 +715,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>frame_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>frame_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>payload_length</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>direction</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -750,28 +749,320 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x1001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Single Cell Data</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>30</v>
+          <t>Cell Relay Control</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>tx</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Relay control (Cell Enable, Cell Select)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>0x1002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cell Charge Select</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Charge parameters (Max Charge Voltage, Current 1 &amp; 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0x1003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cell Charge Control</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Charge control (Charge Enable, Charge Comparator Reset)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0x1004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Cell Discharge Control</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Discharge control (Discharge Enable, Discharge Comparator Reset)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0x1005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cell Data</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>rx</t>
         </is>
       </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Simulink Byte Pack Output</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Cell Voltages &amp; Temperatures</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0x1006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Cell Discharge Select</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>tx</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Discharge load selection (Discharge Load 1..4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0x2000</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Board Parameters</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>rx</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Board Ambient &amp; System Voltages</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0x3000</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Algorithm Faults</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>rx</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Algorithm Fault Flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0x4000</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Protection Threshold</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>rx</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Protection Threshold Limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0x5000</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Estimation Values</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>rx</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>SOC Estimation Values</t>
         </is>
       </c>
     </row>
@@ -786,76 +1077,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id_or_address</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>signal_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>data_type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>count</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>byte_order</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>scale</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>offset</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>group</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>read_write</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>min_value</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>max_value</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
@@ -864,7 +1155,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x1005</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -877,19 +1168,25 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>1</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -906,14 +1203,21 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N2" t="b">
-        <v>1</v>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Cell Terminal Voltage</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x1005</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -926,19 +1230,25 @@
           <t>int16</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>1</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -955,14 +1265,21 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N3" t="b">
-        <v>1</v>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Cell Current</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x1005</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -975,19 +1292,25 @@
           <t>int16</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>1</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1004,14 +1327,21 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N4" t="b">
-        <v>1</v>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Terminal Temp</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x1005</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1024,19 +1354,25 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>1</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1053,14 +1389,21 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N5" t="b">
-        <v>1</v>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Surface Temp</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x2000</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1073,19 +1416,25 @@
           <t>int16</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>1</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1094,7 +1443,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Board Parameters</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1102,14 +1451,21 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N6" t="b">
-        <v>1</v>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Ambient Temp</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x2000</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1122,19 +1478,25 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>1</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1143,7 +1505,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Board Parameters</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1151,14 +1513,21 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N7" t="b">
-        <v>1</v>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Charger Voltage</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x2000</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1171,19 +1540,25 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>1</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1192,7 +1567,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Board Parameters</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1200,19 +1575,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N8" t="b">
-        <v>1</v>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Load Voltage</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x3000</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OVc</t>
+          <t>Faults</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1220,23 +1602,34 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>1</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Bitfields</t>
+        </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Algorithm Faults</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1244,19 +1637,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N9" t="b">
-        <v>1</v>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Fault Flags</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x4000</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>UVc</t>
+          <t>OVc</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1264,23 +1664,34 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>1</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Protection Threshold</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1288,19 +1699,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N10" t="b">
-        <v>1</v>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Over-Voltage Limit</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x4000</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OCc</t>
+          <t>UVc</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1308,23 +1726,34 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>1</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F11" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Protection Threshold</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1332,19 +1761,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N11" t="b">
-        <v>1</v>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Under-Voltage Limit</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x4000</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OCdc</t>
+          <t>OCc</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1352,23 +1788,34 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>1</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F12" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Protection Threshold</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1376,19 +1823,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N12" t="b">
-        <v>1</v>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Over-Current Charge Limit</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x4000</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OTc</t>
+          <t>OCdc</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1396,23 +1850,34 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>1</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F13" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Protection Threshold</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1420,19 +1885,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N13" t="b">
-        <v>1</v>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Over-Current Discharge Limit</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x4000</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>UTc</t>
+          <t>OTc</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1440,23 +1912,34 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>1</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Protection Threshold</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1464,19 +1947,26 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N14" t="b">
-        <v>1</v>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Over-Temp Limit</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x4000</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>OCV_SOC</t>
+          <t>UTc</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1484,28 +1974,34 @@
           <t>uint16</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>1</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>0.001</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Cell Data</t>
+          <t>Protection Threshold</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1513,57 +2009,139 @@
           <t>R</t>
         </is>
       </c>
-      <c r="N15" t="b">
-        <v>1</v>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Under-Temp Limit</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x1000</t>
+          <t>0x5000</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>OCV_SOC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>uint16</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Estimation Values</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Open-Circuit Voltage SOC</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0x5000</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>CC_SOC</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>uint16</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>little</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Cell Data</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Estimation Values</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="N16" t="b">
-        <v>1</v>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Coulomb Counting SOC</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1577,38 +2155,230 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>id_or_address</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>signal_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>bit_index</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>label</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>active_text</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>inactive_text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0x3000</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Faults</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Overvoltage Fault</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>FAULT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>0x3000</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Faults</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Undervoltage Fault</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FAULT</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0x3000</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Faults</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Overcurrent Charge Fault</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>FAULT</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0x3000</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Faults</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Overcurrent Discharge Fault</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>FAULT</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0x3000</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Faults</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Overtemperature Fault</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>FAULT</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0x3000</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Faults</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Undertemperature Fault</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>FAULT</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -1700,33 +2470,148 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>command_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>id_or_address</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>payload_hex</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>enabled</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cell Relay Control</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0x1001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Relay control (Cell Enable, Cell Select)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cell Charge Select</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x1002</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Charge parameters (Max Charge Voltage, Current 1 &amp; 2)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cell Charge Control</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x1003</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Charge control (Charge Enable, Charge Comparator Reset)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cell Discharge Control</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0x1004</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Discharge control (Discharge Enable, Discharge Comparator Reset)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cell Discharge Select</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0x1006</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Discharge load selection (Discharge Load 1..4)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -1741,58 +2626,734 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>command_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>signal_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>data_type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>byte_order</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>scale</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>offset</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>min_value</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>max_value</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>default</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cell Relay Control</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Cell Enable</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cell Relay Control</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cell Select</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Cell Charge Select</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Max Charge Voltage</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cell Charge Select</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Max Charge Current 1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cell Charge Select</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Max Charge Current 2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cell Charge Control</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Charge Enable</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cell Charge Control</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Charge Comparator Reset</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cell Discharge Control</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Discharge Enable</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Cell Discharge Control</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Discharge Comparator Reset</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cell Discharge Select</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Discharge Load 1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cell Discharge Select</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Discharge Load 2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Cell Discharge Select</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Discharge Load 3</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Cell Discharge Select</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Discharge Load 4</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>little</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>

</xml_diff>